<commit_message>
Update the planning documents' build status to 29 Oct
The roadmap phases, the 15 modules and the contract spreadsheet now
show what is built today (backend, content portal, staging, server
quizzes, progress, economy, leagues and Ask AI through the server),
with matching status colours and a change-log entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -708,7 +708,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Build status (27 Oct 2026)</t>
+          <t>Build status (29 Oct 2026)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Design system (Terracotta x Sand theme) and learner user flows exist in the app. Still needed: PRD sign-off, source policy, data dictionary, OpenAPI skeleton, backend stack choice.</t>
+          <t>Design system (Terracotta x Sand) and learner flows exist. Backend stack chosen (NestJS + Postgres), OpenAPI contract in backend/openapi.json. Still needed: PRD sign-off, source policy, data dictionary.</t>
         </is>
       </c>
     </row>
@@ -820,14 +820,14 @@
           <t>All clients authenticate against staging</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Partly done</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>Flutter app shell done. No auth, backend, environments, CI/CD or portal shell yet. Empty backend/ and cms/ folders created in the repo.</t>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Mostly done</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>Learner and staff sign-in with roles, database migrations, CI on every push (backend, portal, app), a staging server with HTTPS and nightly database backups, standard API errors, and the app and portal shells. Still missing: staff management pages, analytics and crash reporting.</t>
         </is>
       </c>
     </row>
@@ -877,14 +877,14 @@
           <t>Reviewed sample pack appears in app</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>Not started. The 108 existing questions (with 5 translations) can be the first sample pack once the pipeline exists.</t>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Partly done</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log. The 108 starter questions are imported. Still missing: taxonomy pages, sources and validity dates on the questions, CSV import.</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Learner screens are built and tested offline (discovery, quiz, explanations, results, progress). Still needed: published content from the API, server scoring, bookmarks, mistake review, reports.</t>
+          <t>Quizzes run on the server: it picks the questions, keeps the answer keys and scores (including exam minus marks). Results, XP, stars, streak, coins, energy and settings are saved to the account. Still missing: bookmarks, mistake review, report-a-question.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Not started (38 automated tests exist for the offline app).</t>
+          <t>Not started. Automated tests exist: 37 unit and 63 API tests for the backend, 40 for the app.</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>Nothing yet.</t>
+          <t>Nothing yet. A staging server is running for testing (staging-api / staging-cms.deepwebstudio.dev).</t>
         </is>
       </c>
     </row>
@@ -1105,14 +1105,14 @@
           <t>Feature tied to measured learner need</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
-        <is>
-          <t>Done in app (offline)</t>
-        </is>
-      </c>
-      <c r="K8" s="9" t="inlineStr">
-        <is>
-          <t>Ahead of plan on the device: streaks, daily challenge, leagues, 6 languages. Reminders and server-backed engagement not done.</t>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Partly done</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Ahead of plan: streaks with freezes, Daily Docket, exam modes and real weekly leagues (on the server, topped up with practice players), 6 app languages. Still missing: push reminders, spaced repetition, language packs for quiz content.</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>Ask AI chat prototype and a demo premium paywall (no real payments).</t>
+          <t>Ask AI answers through the server with Azure OpenAI (gpt-5.4-mini), 5 free a day; no key in the app. Demo premium only (no real payments). Still missing: answers grounded in approved sources with citations.</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Build status (27 Oct 2026)</t>
+          <t>Build status (29 Oct 2026)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -1303,14 +1303,14 @@
           <t>Server-side permissions; session expiry handled</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="inlineStr">
-        <is>
-          <t>The app keeps a local profile only (name, persona, daily goal, language) on the device. No sign-in, roles or backend yet.</t>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>Email and password sign-in for learners and staff, short-lived access tokens with rotating refresh tokens (reuse detected), roles checked on every request, sign-in rate limit per client. Accounts carry XP, coins and settings across phones.</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>App: Explore Law home, Core Laws list and a Journey map of 6 chapters x 3 levels, from a catalog built into the app. No taxonomy API, no CMP, no search or filters (search opens Ask AI).</t>
+          <t>Subjects, topics and acts in the database, served by GET /v1/taxonomy and the quiz catalog; the app maps its 6 chapters to subjects. Still missing: portal pages to manage the taxonomy, search and filters.</t>
         </is>
       </c>
     </row>
@@ -1417,14 +1417,14 @@
           <t>Cannot publish incomplete or unreviewed content</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>The 108 questions are a JSON file bundled in the app. No drafts, review, versions or publishing.</t>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Content Management Portal: create and edit drafts, submit, request changes, approve (reviewer cannot be the author or an editor), publish, revise, retire. Published versions are fixed; every step is in the audit log. 108 starter questions imported.</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Every question has an explanation and a provision reference (e.g. "Article 394, Constitution of India"). No source URL, verified date, validity dates, reviewer or versions.</t>
+          <t>Questions have fields for source title and URL, provision reference and valid-from / valid-to dates, and only questions in force today reach learners. Still missing: sources and dates filled in on the 108 questions, so they can pass real review (on staging they were published unreviewed).</t>
         </is>
       </c>
     </row>
@@ -1533,12 +1533,12 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Done in app (offline)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
-          <t>Four quiz modes: Case Path (level map), Daily Docket (daily challenge), Moot Court Duel and Exam Chamber, with difficulty, question counts and timers. The device picks the questions, not the server.</t>
+          <t>GET /v1/quizzes lists topics with published questions in force; four modes (Case Path, Daily Docket, Duel, Exam Chamber) with question counts, difficulty and the daily set chosen by the server.</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Done in app (offline)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
         <is>
-          <t>Start, answer, explanation and result work end to end, but scoring runs on the device and the answer keys ship inside the app. The plan requires server-side scoring, so this must move to the backend.</t>
+          <t>The server starts the quiz, picks and shuffles the questions, keeps the answer keys, times each answer and scores it, including exam minus marks (+1 / −0.25). Answers are explained after they are final (practice) or after submit (exam). No answer keys in the app.</t>
         </is>
       </c>
     </row>
@@ -1647,12 +1647,12 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Done in app (offline)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>Result screen, stars, XP, Journey progress and stats. Saved on the device only: no attempt history API and no sync across devices.</t>
+          <t>Results with server-worked stars, XP, streak and coins; GET /v1/me/progress and attempt history; progress follows the account to any phone. Real weekly leagues with promotion and demotion.</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>No question bookmarks or mistake notebook yet (Exam Chamber shows a review at the end only). Bookmarks exist for Legal Updates articles only.</t>
+          <t>No question bookmarks or mistake review yet (Exam Chamber shows a review at the end only). Bookmarks exist for Legal Updates articles only.</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>No import or export yet.</t>
+          <t>No CSV import or export yet; the seed script imports the starter questions.</t>
         </is>
       </c>
     </row>
@@ -1816,14 +1816,14 @@
           <t>Permission matrix and audit tests pass</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>No admin portal or admin APIs yet.</t>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Partly done</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>Roles (admin, editor, reviewer, publisher, learner) are enforced in the API and the portal, and actions are audit-logged. Still missing: pages to manage staff accounts and roles.</t>
         </is>
       </c>
     </row>
@@ -1987,14 +1987,14 @@
           <t>Safe language fallback; translated legal content reviewed</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>Done in app (offline)</t>
-        </is>
-      </c>
-      <c r="K14" s="9" t="inlineStr">
-        <is>
-          <t>UI and all 108 questions in 6 languages (English, Hindi, Tamil, Telugu, Kannada, Malayalam), language picker, English fallback. Newest UI strings are English-only; translated content has no legal review; accessibility not audited.</t>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Partly done</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>App UI in 6 languages (English, Hindi, Tamil, Telugu, Kannada, Malayalam) with English fallback. Quiz content is English only on the server for now; the newest screens are English only; translated content has no legal review; accessibility not audited.</t>
         </is>
       </c>
     </row>
@@ -2044,14 +2044,14 @@
           <t>Opt-out respected; jobs timezone-aware and deduplicated</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>Done in app (offline)</t>
-        </is>
-      </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>Streaks with freezes and milestones, Daily Docket daily challenge, energy, XP, weekly leagues and leaderboard, all on the device (league rivals are simulated). No push reminders, preferences API or server jobs.</t>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Partly done</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Streaks with freezes and milestones, Daily Docket, energy, coins and real weekly leagues all run on the server. Still missing: push reminders, notification preferences, scheduled jobs.</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>Ask AI chat exists: it calls Claude directly with a key built into the app, or answers offline. No grounding or citations. The roadmap puts AI in P7 and keeps unreviewed AI answers out of the first release; the built-in key must not ship.</t>
+          <t>Ask AI answers through POST /v1/chat on the server with Azure OpenAI (gpt-5.4-mini), 5 answers a day free; the key stays on the server. Still missing: answers grounded in approved sources, citations, an evaluation set, and legal review of AI answers.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4885,6 +4885,33 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1.0.2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status (Roadmap, Module Register) to 29 Oct 2026: NestJS backend, Content Management Portal, staging server, server-side quizzes, scoring, progress, economy and weekly leagues, and Ask AI through the server.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add sources and dates to the starter questions; link them in the app
Each of the 108 starter questions now carries a researched source: the
official text (Gazette, India Code, Legislative Department, PIB or
Supreme Court), the citation, the date its answer became law, and a note
for the reviewer on how sure the research is. Two DPDP Act questions
only become valid on 13 May 2027, when those sections start.

The seed brings these in without skipping review: drafts get the source
where they have none, and questions published without review get a new
draft revision for a reviewer to approve. Nothing is published.

Learners see a "Read the official text" link under each explanation in
the quiz, the results review and the Review page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log. The 108 starter questions are imported. Still missing: taxonomy pages, sources and validity dates on the questions, CSV import.</t>
+          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log. The 108 starter questions are imported and now carry researched sources, official links and validity dates, waiting for legal review. Still missing: taxonomy pages, staff account pages, CSV import, and a real reviewer signing off a sample pack.</t>
         </is>
       </c>
     </row>
@@ -934,14 +934,14 @@
           <t>Scoring and content parity tests pass</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Partly done</t>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Mostly done</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Quizzes run on the server: it picks the questions, keeps the answer keys and scores (including exam minus marks). Results, XP, stars, streak, coins, energy and settings are saved to the account. Still missing: bookmarks, mistake review, report-a-question.</t>
+          <t>Quizzes run on the server: it picks the questions, keeps the answer keys and scores (including exam minus marks). Results, XP, stars, streak, coins, energy and settings are saved to the account. Saved questions, mistake review and report-a-question are built, and each explanation links to its official source. Still missing: QA sign-off of the learner journey on staging.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Not started. Automated tests exist: 37 unit and 63 API tests for the backend, 40 for the app.</t>
+          <t>Not started. Automated tests exist: 38 unit and 76 API tests for the backend, 41 for the app.</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>Questions have fields for source title and URL, provision reference and valid-from / valid-to dates, and only questions in force today reach learners. Still missing: sources and dates filled in on the 108 questions, so they can pass real review (on staging they were published unreviewed).</t>
+          <t>Questions have source title and URL, citation, provision reference and valid-from / valid-to dates, and only questions in force today reach learners. The app shows the source under each explanation with a link to the official text. All 108 starter questions now carry a researched source (official Gazette, India Code, Legislative Department, PIB or Supreme Court links for 105 of them) and the date each answer became correct; the seed puts them into draft revisions for review. Still missing: legal review of those drafts (on staging the questions were first published unreviewed). Two DPDP Act questions only become valid on 13 May 2027, when those sections come into force.</t>
         </is>
       </c>
     </row>
@@ -1702,14 +1702,14 @@
           <t>Bookmarks sync; attempts retain historical question version</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>No question bookmarks or mistake review yet (Exam Chamber shows a review at the end only). Bookmarks exist for Legal Updates articles only.</t>
+          <t>Learners save questions (kept on the account) and see a mistakes list: questions whose latest final answer was wrong, which leave the list when answered right later. Mistake practice is free and earns XP. Review card on Home and a Review page (Mistakes / Saved); saved and mistake items show the version the learner answered.</t>
         </is>
       </c>
     </row>
@@ -1930,14 +1930,14 @@
           <t>Report never directly edits live content</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Mostly done</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>No "report this question" flow yet.</t>
+          <t>Learners report a question from its explanation or the results review (reason + comment, 20 a day). Staff see and close reports in the portal (Reports page, open reports on each question page, urgent reasons first, audit-logged); a report never changes content. Still missing: telling the reporter the outcome (needs M14).</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4912,6 +4912,33 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1.0.3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: researched sources and validity dates on the 108 starter questions (M04), source links in the app, saved questions and mistake review (M08), report-a-question (M12); P3 mostly done.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Import and export questions as CSV or Excel files
Editors check a file first (nothing is saved; each row's result names
the column and the reason), then import the valid new rows. Imports
only ever create drafts. Rows already in the bank are skipped, repeats
inside a file fail, and the same file cannot be imported twice. Each
import keeps a report.

The question list exports CSV or Excel in the same columns, so a file
can be edited and imported back. Planning documents mark M09 done.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log. The 108 starter questions are imported and now carry researched sources, official links and validity dates, waiting for legal review. Still missing: taxonomy pages, staff account pages, CSV import, and a real reviewer signing off a sample pack.</t>
+          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log, bulk submit / approve / publish, and CSV / Excel import (drafts only, with a test run and row-level errors) and export. The 108 starter questions carry researched sources, official links and validity dates, waiting for legal review. Still missing: taxonomy pages, staff account pages, and a real reviewer signing off a sample pack.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Not started. Automated tests exist: 38 unit and 76 API tests for the backend, 41 for the app.</t>
+          <t>Not started. Automated tests exist: 65 unit and 83 API tests for the backend, 41 for the app.</t>
         </is>
       </c>
     </row>
@@ -1759,14 +1759,14 @@
           <t>Imports create drafts only; row errors are actionable</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>No CSV import or export yet; the seed script imports the starter questions.</t>
+          <t>Content Management Portal → Imports: upload a .csv (UTF-8) or .xlsx file of up to 500 questions, check it first (nothing saved; every row's result with column and reason), then import the valid new rows as drafts only. Unknown columns refuse the file; rows already in the bank (same external_ref, or same text in the same topic) are skipped; repeats inside a file fail; the same file can't be imported twice. Each import keeps a saved report. Export to CSV or Excel in the same columns (follows the status and topic filter), so a file can be edited and imported back.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4939,6 +4939,33 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1.0.4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: question import / export (M09 done), bulk submit / approve / publish in the portal; P2 still needs taxonomy and staff pages and a reviewed sample pack.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manage subjects, topics and acts in the content portal
A new Topics page lists every subject with its topics, hidden ones
included, with question counts. Editors add, rename, reorder, show or
hide topics and acts; only admins change subjects. Slugs never change
and topics stay in their subject, because the app and learners'
progress refer to them; new subjects start hidden, and showing or
hiding asks first, saying what changes for learners.

The question list now names hidden topics too, and marks them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -884,7 +884,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log, bulk submit / approve / publish, and CSV / Excel import (drafts only, with a test run and row-level errors) and export. The 108 starter questions carry researched sources, official links and validity dates, waiting for legal review. Still missing: taxonomy pages, staff account pages, and a real reviewer signing off a sample pack.</t>
+          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log, bulk submit / approve / publish, CSV / Excel import (drafts only, with a test run and row-level errors) and export, and a Topics page for subjects, topics and acts. The 108 starter questions carry researched sources, official links and validity dates, waiting for legal review. Still missing: staff account pages, and a real reviewer signing off a sample pack.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Not started. Automated tests exist: 65 unit and 83 API tests for the backend, 41 for the app.</t>
+          <t>Not started. Automated tests exist: 65 unit and 88 API tests for the backend, 41 for the app.</t>
         </is>
       </c>
     </row>
@@ -1360,14 +1360,14 @@
           <t>Only eligible published content is discoverable</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Partly done</t>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Mostly done</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Subjects, topics and acts in the database, served by GET /v1/taxonomy and the quiz catalog; the app maps its 6 chapters to subjects. Still missing: portal pages to manage the taxonomy, search and filters.</t>
+          <t>Subjects, topics and acts in the database, served by GET /v1/taxonomy and the quiz catalog; the app maps its 6 chapters to subjects. Content Management Portal → Topics: add, rename, reorder, show or hide subjects (admins), topics and acts (editors and admins), with question counts; slugs are fixed, topics stay in their subject, new subjects start hidden, and hidden topics keep their questions but leave quizzes. Still missing: learner search and filters in the app, and new subjects in the app (it has its 6 chapters built in).</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Roles (admin, editor, reviewer, publisher, learner) are enforced in the API and the portal, and actions are audit-logged. Still missing: pages to manage staff accounts and roles.</t>
+          <t>Roles (admin, editor, reviewer, publisher, learner) are enforced in the API and the portal, and actions are audit-logged. Taxonomy pages (subjects admin-only), reports, bulk review actions and question import/export are in the portal. Still missing: pages to manage staff accounts and roles.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4966,6 +4966,33 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1.0.5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: Topics page for subjects, topics and acts (M02 mostly done, M10 partly done); P2 still needs staff account pages and a reviewed sample pack.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manage staff accounts with one-time setup links
Admins add staff from a new Staff page; each person gets a one-time
link (valid 7 days) to choose their own password, so nobody else ever
knows it. Admins change roles, disable or enable accounts (which signs
the person out at once) and make a new link for a forgotten password.
Nobody can remove their own admin role, and there is always an active
admin. Only a hash of each link is stored.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -877,14 +877,14 @@
           <t>Reviewed sample pack appears in app</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Partly done</t>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Mostly done</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>Content Management Portal: write, review and publish questions (draft → review → approved → published), fixed published versions, audit log, bulk submit / approve / publish, CSV / Excel import (drafts only, with a test run and row-level errors) and export, and a Topics page for subjects, topics and acts. The 108 starter questions carry researched sources, official links and validity dates, waiting for legal review. Still missing: staff account pages, and a real reviewer signing off a sample pack.</t>
+          <t>Content Management Portal: write, review and publish questions with fixed versions and an audit log; bulk submit / approve / publish; CSV / Excel import (drafts only, with a test run and row-level errors) and export; a Topics page for subjects, topics and acts; and Staff accounts with one-time setup links and role changes. The 108 starter questions carry researched sources, official links and validity dates. Still missing: a real legal reviewer signing off a sample pack on staging (the exit gate).</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Not started. Automated tests exist: 65 unit and 88 API tests for the backend, 41 for the app.</t>
+          <t>Not started. Automated tests exist: 65 unit and 93 API tests for the backend, 41 for the app.</t>
         </is>
       </c>
     </row>
@@ -1816,14 +1816,14 @@
           <t>Permission matrix and audit tests pass</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>Partly done</t>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>Mostly done</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Roles (admin, editor, reviewer, publisher, learner) are enforced in the API and the portal, and actions are audit-logged. Taxonomy pages (subjects admin-only), reports, bulk review actions and question import/export are in the portal. Still missing: pages to manage staff accounts and roles.</t>
+          <t>Roles (admin, editor, reviewer, publisher, analyst, learner) are enforced in the API and the portal, and actions are audit-logged. Content Management Portal → Staff (admins): invite staff with a one-time link to choose their own password, change roles, disable or enable accounts (signs out at once), and issue a new setup link; nobody can remove their own admin role and there is always an active admin. Also in the portal: Topics, Reports, Imports and bulk review actions. Still missing: feature flags and operational settings pages.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4993,6 +4993,33 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1.0.6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: staff accounts with one-time setup links and role changes (M10 mostly done); P2 mostly done, waiting for a reviewed sample pack.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Let learners delete their own account in the app
Settings has a new Delete account row. It explains what goes, asks for
the password and, once the server has deleted the account, clears the
phone and starts again. The API's new route removes the account and the
personal data on it (quiz sessions, wallet, settings, saved questions,
league places, sign-in tokens, the learner's own audit entries). Reports
they sent stay for the editors without their name. Staff accounts are
removed by admins, not by their owners.

Both app stores require deletion from inside the app.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -991,14 +991,14 @@
           <t>UAT and release checklist signed</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Partly done</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Not started. Automated tests exist: 65 unit and 93 API tests for the backend, 41 for the app.</t>
+          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion. Decided: Sentry for crash reporting, our own usage events for analytics, citizens as the beta audience, production hosting later. Still to do: Sentry, usage events and a dashboard, minimum app version, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 65 unit and 97 API tests for the backend, 42 for the app.</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
-          <t>Email and password sign-in for learners and staff, short-lived access tokens with rotating refresh tokens (reuse detected), roles checked on every request, sign-in rate limit per client. Accounts carry XP, coins and settings across phones.</t>
+          <t>Email and password sign-in for learners and staff, short-lived access tokens with rotating refresh tokens (reuse detected), roles checked on every request, sign-in rate limit per client. Accounts carry XP, coins and settings across phones. Staff accounts are managed by admins with one-time setup links. Learners can delete their own account in the app, confirmed with their password: their data is removed and nothing links the deleted account to a person.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5020,6 +5020,33 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>1.0.7</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: P4 started (premium hidden for the beta; learners can delete their own account in the app); M01 done.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Report crashes and errors from the app to Sentry
The app now sends unexpected errors to Sentry when it is built with a
SENTRY_DSN (kept out of the repo, in a git-ignored settings file). Only
errors are sent: no performance traces, screenshots, taps or personal
details. Offline, timeouts and the API's own refusals are ignored;
server errors and unexpected faults are reported.

A debug-only Settings row sends a test error to check the setup. The
Privacy text now matches how the app works today (progress on the
account, crash reports, account deletion), in all six languages.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion. Decided: Sentry for crash reporting, our own usage events for analytics, citizens as the beta audience, production hosting later. Still to do: Sentry, usage events and a dashboard, minimum app version, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 65 unit and 97 API tests for the backend, 42 for the app.</t>
+          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), and a corrected privacy text. Decided: our own usage events for analytics, citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, usage events and a dashboard, minimum app version, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 65 unit and 97 API tests for the backend, 44 for the app.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5047,6 +5047,33 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>1.0.8</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: crash reporting (Sentry) in the app, corrected privacy text; P4 partly done.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add usage analytics and an Analytics page to the content portal
Admins and analysts see learners, who is active today, this week and
this month, a daily series, 1-, 7- and 30-day retention, quizzes by
mode, and the most-missed questions with open reports. The numbers are
calculated from what the app already records, so nothing extra is
tracked, except one small marker: the app now tells the server once a
day that it was opened, which retention needs. The marker goes when a
learner deletes their account.

The Privacy text mentions it, in all six languages. No names or emails
appear on the page.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), and a corrected privacy text. Decided: our own usage events for analytics, citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, usage events and a dashboard, minimum app version, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 65 unit and 97 API tests for the backend, 44 for the app.</t>
+          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), usage analytics with a portal dashboard (calculated from existing records), and a corrected privacy text. Decided: citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, minimum app version, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 65 unit and 102 API tests for the backend, 46 for the app.</t>
         </is>
       </c>
     </row>
@@ -1873,14 +1873,14 @@
           <t>Events validated; no secrets or answer keys in telemetry</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Partly done</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>No analytics events or crash reporting yet.</t>
+          <t>Usage analytics are done without a separate event stream: the Content Management Portal's Analytics page (admins and analysts) is calculated from what the app already records, plus a once-a-day note that a learner opened the app. It shows learners, activity today / 7 / 30 days, a daily series, 1-, 7- and 30-day retention, quizzes by mode, the most-missed questions and open reports. No names or emails; a learner's data goes when they delete their account. Crash reporting with Sentry is in the app. Still missing: Sentry for the API and the portal, error alerts, and the screen-level events the sheet lists (result viewed).</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5074,6 +5074,33 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>1.0.9</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: usage analytics and the portal Analytics page (M11 partly done); P4 further along.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tell app builds that are too old to update
The API gives the minimum allowed app version at GET /v1/app-config
(MIN_APP_VERSION, APP_UPDATE_URL). The app asks at start and on resume and,
if older, shows only an update screen. Offline never blocks anyone.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), usage analytics with a portal dashboard (calculated from existing records), and a corrected privacy text. Decided: citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, minimum app version, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 65 unit and 102 API tests for the backend, 46 for the app.</t>
+          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), usage analytics with a portal dashboard (calculated from existing records), a minimum app version check (old builds are told to update), and a corrected privacy text. Decided: citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 67 unit and 104 API tests for the backend, 55 for the app.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5101,6 +5101,33 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>1.0.10</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: minimum app version check (old builds are told to update); P4 further along.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Translate the English-only screens into the five other languages
111 texts per language (onboarding, sign-in, Explore Law, Review, reports,
quiz errors) now exist in Hindi, Tamil, Telugu, Kannada and Malayalam. A test
fails if a language misses a text or changes a placeholder.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), usage analytics with a portal dashboard (calculated from existing records), a minimum app version check (old builds are told to update), and a corrected privacy text. Decided: citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, translations of English-only screens, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 67 unit and 104 API tests for the backend, 55 for the app.</t>
+          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), usage analytics with a portal dashboard (calculated from existing records), a minimum app version check (old builds are told to update), translations of the English-only screens into five languages (to be read by native speakers), and a corrected privacy text. Decided: citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 67 unit and 104 API tests for the backend, 60 for the app.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5128,6 +5128,33 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1.0.11</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: translations of the English-only screens into Hindi, Tamil, Telugu, Kannada and Malayalam (machine drafts, native review needed); P4 further along.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Report crashes from the API and the content portal to Sentry
Errors only, same privacy rules as the app: no user, request data,
breadcrumbs or traces. Database error text after 'params:' and the query
string and #fragment of page addresses are removed before sending. Keys come
from the server's .env (API_SENTRY_DSN, PORTAL_SENTRY_DSN).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/planning/03_Integration_Content_Contract.xlsx
+++ b/docs/planning/03_Integration_Content_Contract.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
-          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting in the app with Sentry (errors only, no personal details), usage analytics with a portal dashboard (calculated from existing records), a minimum app version check (old builds are told to update), translations of the English-only screens into five languages (to be read by native speakers), and a corrected privacy text. Decided: citizens as the beta audience, production hosting later. Still to do: Sentry for the API and the portal, accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 67 unit and 104 API tests for the backend, 60 for the app.</t>
+          <t>Started. Done: premium hidden for the beta (the app and the API), in-app account deletion, crash reporting with Sentry in the app, the API and the portal (errors only, no personal details), usage analytics with a portal dashboard (calculated from existing records), a minimum app version check (old builds are told to update), translations of the English-only screens into five languages (to be read by native speakers), and a corrected privacy text. Decided: citizens as the beta audience, production hosting later. Still to do: accessibility and dark-mode check, shared sign-in rate limit, key rotation, store preparation. Automated tests: 71 unit and 104 API tests for the backend, 60 for the app.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5155,6 +5155,33 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>1.0.12</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Updated build status: crash reporting with Sentry now also in the API and the content portal (errors only); P4 further along.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Pending team review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>